<commit_message>
updates on bill of materials
</commit_message>
<xml_diff>
--- a/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
+++ b/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidstjohn/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidstjohn/Desktop/Edge-Computing-Power-Management-Development-Kit/hardware/v0.1.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22BA6815-478F-C041-AF41-EFE06DCF12A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B173B3A-1B9E-E44A-9A65-8935D9274B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PATCH 6.0" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="PATCH 8.0A" sheetId="5" r:id="rId5"/>
     <sheet name="PATCH 8.0D" sheetId="6" r:id="rId6"/>
     <sheet name="BOM" sheetId="7" r:id="rId7"/>
+    <sheet name="Bill of Materials" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="154">
   <si>
     <t xml:space="preserve">Part </t>
   </si>
@@ -441,13 +442,79 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/molex/1050170001/2350832?s=N4IgTCBcDaIIwAYCsC4HYC0DtxAXQF8g</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Quantity per Board</t>
+  </si>
+  <si>
+    <t>Total Quantity</t>
+  </si>
+  <si>
+    <t>Unit Cost</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Mfr: #</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Vendor 2</t>
+  </si>
+  <si>
+    <t>100 nF capacitor (0603)</t>
+  </si>
+  <si>
+    <t>No CR1220 in main lab battery drawer.</t>
+  </si>
+  <si>
+    <t>We already have LiPO batteries and connections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.rocelec.com/part/01t4w00000PPv4UAAT-PCF8523T1118?utm_term=&amp;utm_campaign=USA+-+PMAX&amp;utm_source=adwords&amp;utm_medium=ppc&amp;hsa_net=adwords&amp;hsa_tgt=&amp;hsa_ad=&amp;hsa_acc=2274246953&amp;hsa_grp=&amp;hsa_mt=&amp;hsa_cam=19547754453&amp;hsa_kw=&amp;hsa_ver=3&amp;hsa_src=x&amp;gad_source=4&amp;gad_campaignid=19547755830&amp;gbraid=0AAAAADfiOy4l2s7LtXtyp4aJxaq1bq5_A&amp;gclid=CjwKCAjw8arQBhB9EiwAfIKdQq3H62HP9EGlikIHKTUOl6LLbTMsnXpAQsdRDmIj-SLJR3Y_Lyf35xoCwh4QAvD_BwE </t>
+  </si>
+  <si>
+    <t>This part is no longer being manufactured. It was hard to find a vendor</t>
+  </si>
+  <si>
+    <t>Vendo 1 (digikey)</t>
+  </si>
+  <si>
+    <t>ABS05-32.768KHZ-6-T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.sparkfun.com/jst-right-angle-connector-through-hole-2-pin.html </t>
+  </si>
+  <si>
+    <t>Coin Cell battery</t>
+  </si>
+  <si>
+    <t>These are quite expensive. We already have one of these.</t>
+  </si>
+  <si>
+    <t>C0603C220J5GACTU</t>
+  </si>
+  <si>
+    <t>RC0603FR-0710KL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -498,6 +565,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF444444"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -520,7 +601,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -565,9 +646,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3051,7 +3133,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D2AD354-F000-43EA-9051-5CE410C07359}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
@@ -3260,7 +3342,7 @@
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="3" t="s">
         <v>122</v>
       </c>
       <c r="H8" s="3"/>
@@ -3599,6 +3681,617 @@
     <hyperlink ref="C8" r:id="rId21" xr:uid="{E3F21928-8DA8-3841-8335-32FEA84720BE}"/>
     <hyperlink ref="E7" r:id="rId22" xr:uid="{CE7992D0-B119-6B4C-B345-9C25EF9FE2C3}"/>
     <hyperlink ref="E11" r:id="rId23" xr:uid="{B5C99938-5A12-5C43-B38A-88FEEC725884}"/>
+    <hyperlink ref="C13" r:id="rId24" xr:uid="{0F3CB72E-BCDA-134F-BD19-312DB2E785FD}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55933E0B-84C2-874E-A805-F8397A851F43}">
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="54.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="51.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" s="16">
+        <v>3</v>
+      </c>
+      <c r="F2" s="18">
+        <v>4.16</v>
+      </c>
+      <c r="G2" s="18">
+        <f>E2*F2</f>
+        <v>12.48</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="J2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="16">
+        <v>3</v>
+      </c>
+      <c r="F3" s="20">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="G3" s="20">
+        <f>E3*F3</f>
+        <v>1.7399999999999998</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="16">
+        <v>3</v>
+      </c>
+      <c r="F4" s="19">
+        <v>7.01</v>
+      </c>
+      <c r="G4" s="18">
+        <f t="shared" ref="G4:G20" si="0">E4*F4</f>
+        <v>21.03</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" s="16">
+        <v>3</v>
+      </c>
+      <c r="F5" s="20">
+        <v>0.75770000000000004</v>
+      </c>
+      <c r="G5" s="20">
+        <f t="shared" si="0"/>
+        <v>2.2731000000000003</v>
+      </c>
+      <c r="H5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="K5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="16">
+        <v>3</v>
+      </c>
+      <c r="F6" s="20">
+        <v>1.28</v>
+      </c>
+      <c r="G6" s="18">
+        <f t="shared" si="0"/>
+        <v>3.84</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="J6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B7" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7">
+        <v>9749</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="16">
+        <v>5</v>
+      </c>
+      <c r="F7" s="19">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G7" s="20">
+        <f t="shared" si="0"/>
+        <v>5.5</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" s="16">
+        <v>5</v>
+      </c>
+      <c r="F8" s="19">
+        <v>1.06</v>
+      </c>
+      <c r="G8" s="18">
+        <f t="shared" si="0"/>
+        <v>5.3000000000000007</v>
+      </c>
+      <c r="H8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="J8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>3000</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="16">
+        <v>3</v>
+      </c>
+      <c r="F9" s="19">
+        <v>0.4</v>
+      </c>
+      <c r="G9" s="20">
+        <f t="shared" si="0"/>
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>11574</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16">
+        <v>2</v>
+      </c>
+      <c r="F10" s="19">
+        <v>31.88</v>
+      </c>
+      <c r="G10" s="18">
+        <f t="shared" si="0"/>
+        <v>63.76</v>
+      </c>
+      <c r="H10" t="s">
+        <v>151</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="J10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11">
+        <v>1660</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" s="16">
+        <v>3</v>
+      </c>
+      <c r="F11" s="19">
+        <v>1.95</v>
+      </c>
+      <c r="G11" s="20">
+        <f t="shared" si="0"/>
+        <v>5.85</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="J11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B12" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12">
+        <v>3814</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" s="16">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19">
+        <v>0.75</v>
+      </c>
+      <c r="G12" s="18">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>144</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B13" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13">
+        <v>1050170001</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" s="16">
+        <v>3</v>
+      </c>
+      <c r="F13" s="19">
+        <v>0.92</v>
+      </c>
+      <c r="G13" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7600000000000002</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="J13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B14" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="16">
+        <v>10</v>
+      </c>
+      <c r="F14" s="19">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="G14" s="18">
+        <f t="shared" si="0"/>
+        <v>0.21000000000000002</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="J14" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B15" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" s="16">
+        <v>10</v>
+      </c>
+      <c r="F15" s="19">
+        <v>0.03</v>
+      </c>
+      <c r="G15" s="20">
+        <f t="shared" si="0"/>
+        <v>0.3</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="J15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="16">
+        <v>10</v>
+      </c>
+      <c r="F16" s="19">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="G16" s="18">
+        <f t="shared" si="0"/>
+        <v>0.37</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="J16" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" t="s">
+        <v>152</v>
+      </c>
+      <c r="D17" t="s">
+        <v>115</v>
+      </c>
+      <c r="E17" s="16">
+        <v>10</v>
+      </c>
+      <c r="F17" s="19">
+        <v>7.1999999999999995E-2</v>
+      </c>
+      <c r="G17" s="20">
+        <f t="shared" si="0"/>
+        <v>0.72</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="J17" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E18" s="16">
+        <v>10</v>
+      </c>
+      <c r="F18" s="19">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="G18" s="18">
+        <f t="shared" si="0"/>
+        <v>2.8499999999999996</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="J18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B19" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" t="s">
+        <v>115</v>
+      </c>
+      <c r="E19" s="16">
+        <v>10</v>
+      </c>
+      <c r="F19" s="19">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="G19" s="20">
+        <f t="shared" si="0"/>
+        <v>0.34</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" t="s">
+        <v>153</v>
+      </c>
+      <c r="D20" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" s="14">
+        <v>10</v>
+      </c>
+      <c r="F20" s="19">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="G20" s="18">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="J20" t="s">
+        <v>115</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{784743AC-1CA9-2E4A-B45E-71C10508EDE0}"/>
+    <hyperlink ref="I17" r:id="rId2" xr:uid="{151EA8BB-FCA8-4242-89E5-22A6BAA0DF4A}"/>
+    <hyperlink ref="I12" r:id="rId3" xr:uid="{E869A8A3-1E39-324F-B9EB-AEB400CA1C48}"/>
+    <hyperlink ref="I4" r:id="rId4" xr:uid="{2FAD39F5-B682-8846-97F2-096DB73A8DB6}"/>
+    <hyperlink ref="I15" r:id="rId5" xr:uid="{D3EC366E-078B-CC4B-81D0-A5AF54E25A6F}"/>
+    <hyperlink ref="I14" r:id="rId6" xr:uid="{9FA52737-046B-F94E-BD9A-848A25C977F8}"/>
+    <hyperlink ref="I10" r:id="rId7" display="https://www.digikey.com/en/products/detail/sparkfun-electronics/SEN-11574/5762397?utm_adgroup=Gadgets%2C%20Gizmos&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=Shopping_Product_Maker%2FDIY%2C%20Educational_NEW&amp;utm_term=&amp;utm_content=Gadgets%2C%20Gizmos&amp;gclid=CjwKCAjw9pGjBhB-EiwAa5jl3J_1Q2A72ybnR56Rk9sAeqpF2Q-o0ZcV8a4OguEqfE4Nv3m8NDQ9yxoCtdIQAvD_BwE" xr:uid="{0055941C-0675-8D46-9C92-81B8DB6E2429}"/>
+    <hyperlink ref="I3" r:id="rId8" xr:uid="{E36B3917-034D-4546-AC9A-28C3CFF43C58}"/>
+    <hyperlink ref="I16" r:id="rId9" xr:uid="{D717E9B0-7B3E-914B-A144-1A9E7938A3E3}"/>
+    <hyperlink ref="I19" r:id="rId10" xr:uid="{1BFBF5F8-A755-C040-B919-854624B1561B}"/>
+    <hyperlink ref="I18" r:id="rId11" xr:uid="{E795A01A-E799-B04D-A5E2-5F82BC618D8D}"/>
+    <hyperlink ref="I20" r:id="rId12" xr:uid="{D54F72EC-6324-934D-86F6-CAC1B1BEB84D}"/>
+    <hyperlink ref="I8" r:id="rId13" xr:uid="{50120389-F8DF-DF40-9233-9A6B37C405C5}"/>
+    <hyperlink ref="I13" r:id="rId14" xr:uid="{27B8C719-388A-7745-9A17-B4D105976BCB}"/>
+    <hyperlink ref="I5" r:id="rId15" xr:uid="{B4A5999F-110E-5F4B-8D7D-E9F98C55BC7F}"/>
+    <hyperlink ref="J5" r:id="rId16" display="https://www.rocelec.com/part/01t4w00000PPv4UAAT-PCF8523T1118?utm_term=&amp;utm_campaign=USA+-+PMAX&amp;utm_source=adwords&amp;utm_medium=ppc&amp;hsa_net=adwords&amp;hsa_tgt=&amp;hsa_ad=&amp;hsa_acc=2274246953&amp;hsa_grp=&amp;hsa_mt=&amp;hsa_cam=19547754453&amp;hsa_kw=&amp;hsa_ver=3&amp;hsa_src=x&amp;gad_source=4&amp;gad_campaignid=19547755830&amp;gbraid=0AAAAADfiOy4l2s7LtXtyp4aJxaq1bq5_A&amp;gclid=CjwKCAjw8arQBhB9EiwAfIKdQq3H62HP9EGlikIHKTUOl6LLbTMsnXpAQsdRDmIj-SLJR3Y_Lyf35xoCwh4QAvD_BwE " xr:uid="{03C51AB2-4B6A-C441-92C2-B793CBDB24A0}"/>
+    <hyperlink ref="I6" r:id="rId17" xr:uid="{1F0504D9-999B-604A-BC8C-1DD58F2649EA}"/>
+    <hyperlink ref="I7" r:id="rId18" xr:uid="{565A1A2A-1FB1-4D4C-A2AD-F6B6C84B766A}"/>
+    <hyperlink ref="J7" r:id="rId19" xr:uid="{14BD23B7-0DF2-9B45-A14B-30760B9BE651}"/>
+    <hyperlink ref="I9" r:id="rId20" xr:uid="{9ADD7A19-15AF-004C-80C5-0F4C51699992}"/>
+    <hyperlink ref="I11" r:id="rId21" xr:uid="{403F295A-2B42-DE4C-8F52-FE0B71B85BF1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
uUpdatesto BOM post order.
</commit_message>
<xml_diff>
--- a/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
+++ b/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidstjohn/Desktop/Edge-Computing-Power-Management-Development-Kit/hardware/v0.1.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Edge-Computing-Power-Management-Development-Kit\hardware\v0.1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB1C7A13-F49B-7C46-AB5B-F69B7FEF11D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14CDE02-5018-45EE-9967-16341E068397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-150" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PATCH 6.0" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="PATCH 8.0D" sheetId="6" r:id="rId6"/>
     <sheet name="BOM" sheetId="8" r:id="rId7"/>
     <sheet name="Orders" sheetId="9" r:id="rId8"/>
-    <sheet name="old BOM" sheetId="7" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="161">
   <si>
     <t xml:space="preserve">Part </t>
   </si>
@@ -343,9 +342,6 @@
     <t>47 uF capacitor (1206)</t>
   </si>
   <si>
-    <t>Kyocera</t>
-  </si>
-  <si>
     <t>F930J476MAA</t>
   </si>
   <si>
@@ -355,9 +351,6 @@
     <t>10 kΩ resistor (0805)</t>
   </si>
   <si>
-    <t>YAGEO</t>
-  </si>
-  <si>
     <t>RC0805FR-0710KL</t>
   </si>
   <si>
@@ -367,30 +360,9 @@
     <t>NCP711ASN330T1G</t>
   </si>
   <si>
-    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/609/CL10A475KP8NNNC_Spec.pdf</t>
-  </si>
-  <si>
-    <t>https://datasheets.kyocera-avx.com/F93.pdf</t>
-  </si>
-  <si>
-    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/609/CL10A105KA8NNNC_Spec.pdf</t>
-  </si>
-  <si>
-    <t>https://yageogroup.com/content/datasheet/asset/file/PYU-RC_GROUP_51_ROHS_L</t>
-  </si>
-  <si>
-    <t>https://www.molex.com/content/dam/molex/molex-dot-com/products/automated/en-us/salesdrawingpdf/105/105017/1050170001_sd.pdf?inline</t>
-  </si>
-  <si>
     <t>Right angle JST connector</t>
   </si>
   <si>
-    <t>PRT-09749</t>
-  </si>
-  <si>
-    <t>https://cdn.sparkfun.com/assets/4/d/3/e/a/JST_Right_Angle_Connector_-_Through-Hole.pdf</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
@@ -400,42 +372,18 @@
     <t xml:space="preserve">https://www.digikey.com/en/products/detail/yageo/RC0603FR-0710KL/726880 </t>
   </si>
   <si>
-    <t>Ordered (Y/N)</t>
-  </si>
-  <si>
-    <t>Quantity to Order (total for 3 boards)</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/panasonic-energy/CR1220/269740</t>
   </si>
   <si>
-    <t>Coin Cell battery (CR1220)</t>
-  </si>
-  <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
     <t>CR1220</t>
   </si>
   <si>
-    <t>5 (no CR1220 in main lab battery drawer)</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/nxp-usa-inc/PCF8523T-1-118/2530422?s=N4IgTCBcDaIAoGEBiAOArGAzAFQPQEYAaffFEAXQF8g</t>
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/abracon-llc/ABS05-32-768KHZ-6-T/15621978?s=N4IgTCBcDaIIICEDKAGArAWgMxgHQHYA2ADgGsAJALw0IwBUQBdAXyA</t>
   </si>
   <si>
-    <t>Alternate Purchase Link (when not available)</t>
-  </si>
-  <si>
-    <t>https://www.sparkfun.com/jst-right-angle-connector-through-hole-2-pin.html</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/sparkfun-electronics/09749/14671658?s=N4IgTCBcDaIAoCUAqBaADATgOwBYMgF0BfIA</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/keystone-electronics/3000/227440</t>
   </si>
   <si>
@@ -475,9 +423,6 @@
     <t>100 nF capacitor (0603)</t>
   </si>
   <si>
-    <t>No CR1220 in main lab battery drawer.</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.rocelec.com/part/01t4w00000PPv4UAAT-PCF8523T1118?utm_term=&amp;utm_campaign=USA+-+PMAX&amp;utm_source=adwords&amp;utm_medium=ppc&amp;hsa_net=adwords&amp;hsa_tgt=&amp;hsa_ad=&amp;hsa_acc=2274246953&amp;hsa_grp=&amp;hsa_mt=&amp;hsa_cam=19547754453&amp;hsa_kw=&amp;hsa_ver=3&amp;hsa_src=x&amp;gad_source=4&amp;gad_campaignid=19547755830&amp;gbraid=0AAAAADfiOy4l2s7LtXtyp4aJxaq1bq5_A&amp;gclid=CjwKCAjw8arQBhB9EiwAfIKdQq3H62HP9EGlikIHKTUOl6LLbTMsnXpAQsdRDmIj-SLJR3Y_Lyf35xoCwh4QAvD_BwE </t>
   </si>
   <si>
@@ -556,15 +501,6 @@
     <t>Total:</t>
   </si>
   <si>
-    <t>These are quite expensive. We already have one of these. Let me know if you have ideas for substitutes.</t>
-  </si>
-  <si>
-    <t>This part is no longer being manufactured. It was hard to find a vendor.</t>
-  </si>
-  <si>
-    <t>We already have LiPO batteries and connections.</t>
-  </si>
-  <si>
     <t>Vendo 1</t>
   </si>
   <si>
@@ -587,6 +523,9 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/jst-sales-america-inc/S2B-PH-K-S/926626?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlg8DtxjqiUDwety2k6cAQ0XJ&amp;gclid=Cj0KCQjwlLDQBhDjARIsAPlIefHomTfTUoZ7D0P94S5mAVF3io454K95fTm66EAoDjt__qy-ohuCJpkaAg9wEALw_wcB</t>
+  </si>
+  <si>
+    <t>This part is no longer being manufactured.</t>
   </si>
 </sst>
 </file>
@@ -596,7 +535,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -634,11 +573,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF333333"/>
-      <name val="Calibri (Body)"/>
     </font>
     <font>
       <sz val="11"/>
@@ -683,7 +617,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -707,30 +641,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <extLst>
@@ -740,6 +661,9 @@
       </extLst>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1073,16 +997,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.83203125" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" customWidth="1"/>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1099,7 +1023,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1116,7 +1040,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1133,7 +1057,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1150,7 +1074,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1167,7 +1091,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1184,7 +1108,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1201,7 +1125,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1218,7 +1142,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1235,7 +1159,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1252,7 +1176,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1269,7 +1193,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -1286,7 +1210,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -1303,7 +1227,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>52</v>
       </c>
@@ -1320,7 +1244,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -1367,18 +1291,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CB212D0-471F-455A-8AB9-B9E0E3E742F2}">
   <dimension ref="A1:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="29.1640625" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="29.140625" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="27.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1407,7 +1331,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -1433,7 +1357,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1459,7 +1383,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1485,7 +1409,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1511,7 +1435,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1534,7 +1458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1554,7 +1478,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1571,7 +1495,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1591,7 +1515,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1611,7 +1535,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -1628,7 +1552,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -1648,7 +1572,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1671,7 +1595,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -1694,7 +1618,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -1720,7 +1644,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>55</v>
       </c>
@@ -1743,7 +1667,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -1766,7 +1690,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
     </row>
   </sheetData>
@@ -1802,17 +1726,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84474A6A-4EB5-47CC-BBC9-C8313FA58B1E}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="19.5" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1835,7 +1759,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -1855,7 +1779,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1875,7 +1799,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1895,7 +1819,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1912,7 +1836,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1932,7 +1856,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1952,7 +1876,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1969,7 +1893,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1989,7 +1913,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2009,7 +1933,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -2026,7 +1950,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -2046,7 +1970,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -2066,7 +1990,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>81</v>
       </c>
@@ -2086,7 +2010,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -2106,7 +2030,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -2158,17 +2082,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B733AAEF-A146-400A-99FA-6712F1F13B2D}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" customWidth="1"/>
-    <col min="5" max="5" width="32.5" customWidth="1"/>
-    <col min="7" max="7" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="32.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2191,7 +2115,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -2211,7 +2135,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2231,7 +2155,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -2251,7 +2175,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2268,7 +2192,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -2288,7 +2212,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -2308,7 +2232,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -2325,7 +2249,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -2345,7 +2269,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2365,7 +2289,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -2382,7 +2306,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -2402,7 +2326,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -2422,7 +2346,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -2442,7 +2366,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -2462,7 +2386,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>55</v>
       </c>
@@ -2482,7 +2406,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2535,16 +2459,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF29EDA0-EA9F-4349-8100-5B6672D54BB2}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
-    <col min="5" max="5" width="28.1640625" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2567,7 +2491,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -2587,7 +2511,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2607,7 +2531,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -2627,7 +2551,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2644,7 +2568,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -2664,7 +2588,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -2684,7 +2608,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -2701,7 +2625,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -2721,7 +2645,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2741,7 +2665,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -2758,7 +2682,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -2778,7 +2702,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>81</v>
       </c>
@@ -2798,7 +2722,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -2818,7 +2742,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>85</v>
       </c>
@@ -2869,16 +2793,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669867F0-F472-4618-8528-C22270E93F2A}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2901,7 +2825,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -2921,7 +2845,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2941,7 +2865,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -2961,7 +2885,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2978,7 +2902,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -2998,7 +2922,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -3018,7 +2942,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -3035,7 +2959,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -3055,7 +2979,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -3075,7 +2999,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -3092,7 +3016,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -3112,7 +3036,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>77</v>
       </c>
@@ -3132,7 +3056,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>81</v>
       </c>
@@ -3152,7 +3076,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
@@ -3172,7 +3096,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>85</v>
       </c>
@@ -3224,75 +3148,75 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55933E0B-84C2-874E-A805-F8397A851F43}">
   <dimension ref="A1:M22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="80" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="51.83203125" customWidth="1"/>
-    <col min="10" max="10" width="29.1640625" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.5703125" customWidth="1"/>
+    <col min="9" max="9" width="51.85546875" customWidth="1"/>
+    <col min="10" max="10" width="29.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>137</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>155</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="19" t="s">
         <v>65</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="13">
         <v>3</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="14">
         <v>4.16</v>
       </c>
-      <c r="G2" s="18">
+      <c r="G2" s="14">
         <f>E2*F2</f>
         <v>12.48</v>
       </c>
@@ -3300,32 +3224,32 @@
         <v>67</v>
       </c>
       <c r="J2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="K2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
-        <v>106</v>
+      <c r="C3" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="13">
         <v>3</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="15">
         <v>0.57999999999999996</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="15">
         <f>E3*F3</f>
         <v>1.7399999999999998</v>
       </c>
@@ -3333,32 +3257,32 @@
         <v>14</v>
       </c>
       <c r="J3" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="K3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>89</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="13">
         <v>3</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="14">
         <v>7.01</v>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="14">
         <f t="shared" ref="G4:G20" si="0">E4*F4</f>
         <v>21.03</v>
       </c>
@@ -3366,350 +3290,341 @@
         <v>91</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="K4" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>93</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="13">
         <v>3</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="15">
         <v>0.75770000000000004</v>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="15">
         <f t="shared" si="0"/>
         <v>2.2731000000000003</v>
       </c>
       <c r="H5" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>179</v>
+        <v>158</v>
       </c>
       <c r="M5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C6" t="s">
-        <v>145</v>
+      <c r="C6" s="3" t="s">
+        <v>127</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="13">
         <v>3</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="15">
         <v>1.28</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="14">
         <f t="shared" si="0"/>
         <v>3.84</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="J6" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="K6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7">
+        <v>145</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="3">
         <v>9749</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="13">
         <v>5</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="14">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="15">
         <f t="shared" si="0"/>
         <v>5.5</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="K7" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" t="s">
-        <v>123</v>
+        <v>128</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="13">
         <v>5</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="14">
         <v>1.06</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="14">
         <f t="shared" si="0"/>
         <v>5.3000000000000007</v>
       </c>
-      <c r="H8" t="s">
-        <v>143</v>
-      </c>
       <c r="I8" s="9" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="J8" t="s">
-        <v>115</v>
-      </c>
-      <c r="K8" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="3">
         <v>3000</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="13">
         <v>3</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="14">
         <v>0.4</v>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="15">
         <f t="shared" si="0"/>
         <v>1.2000000000000002</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="J9" t="s">
-        <v>115</v>
-      </c>
-      <c r="K9" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="3">
         <v>11574</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="13">
         <v>2</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="14">
         <v>31.88</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="14">
         <f t="shared" si="0"/>
         <v>63.76</v>
       </c>
-      <c r="H10" t="s">
-        <v>170</v>
-      </c>
       <c r="I10" s="9" t="s">
         <v>36</v>
       </c>
       <c r="J10" t="s">
-        <v>115</v>
-      </c>
-      <c r="K10" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>147</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="3">
         <v>1660</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="13">
         <v>3</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="14">
         <v>1.95</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="15">
         <f t="shared" si="0"/>
         <v>5.85</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="L11" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="3">
         <v>3814</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="13">
         <v>0</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="14">
         <v>0.75</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="14">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" t="s">
-        <v>172</v>
-      </c>
       <c r="I12" s="9" t="s">
         <v>41</v>
       </c>
       <c r="J12" t="s">
-        <v>115</v>
-      </c>
-      <c r="K12" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="3">
         <v>1050170001</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="13">
         <v>3</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="14">
         <v>0.92</v>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="15">
         <f t="shared" si="0"/>
         <v>2.7600000000000002</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="J13" t="s">
-        <v>115</v>
-      </c>
-      <c r="K13" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>74</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="13">
         <v>10</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="14">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="14">
         <f t="shared" si="0"/>
         <v>0.21000000000000002</v>
       </c>
@@ -3717,32 +3632,32 @@
         <v>75</v>
       </c>
       <c r="J14" t="s">
-        <v>115</v>
-      </c>
-      <c r="K14" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="3" t="s">
         <v>82</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="13">
         <v>10</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="14">
         <v>0.03</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="15">
         <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
@@ -3750,29 +3665,29 @@
         <v>83</v>
       </c>
       <c r="J15" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="3" t="s">
         <v>57</v>
       </c>
       <c r="D16">
         <v>3</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="13">
         <v>10</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="14">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="14">
         <f t="shared" si="0"/>
         <v>0.37</v>
       </c>
@@ -3780,32 +3695,32 @@
         <v>58</v>
       </c>
       <c r="J16" t="s">
-        <v>115</v>
-      </c>
-      <c r="K16" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C17" t="s">
-        <v>147</v>
+      <c r="C17" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="D17">
         <v>2</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="13">
         <v>10</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="14">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="15">
         <f t="shared" si="0"/>
         <v>0.72</v>
       </c>
@@ -3813,126 +3728,126 @@
         <v>88</v>
       </c>
       <c r="J17" t="s">
-        <v>115</v>
-      </c>
-      <c r="K17" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C18" t="s">
-        <v>100</v>
+      <c r="C18" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="13">
         <v>10</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="14">
         <v>0.28499999999999998</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="14">
         <f t="shared" si="0"/>
         <v>2.8499999999999996</v>
       </c>
       <c r="I18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="J18" t="s">
+        <v>106</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="J18" t="s">
-        <v>115</v>
-      </c>
-      <c r="K18" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>154</v>
-      </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="C19" t="s">
-        <v>104</v>
       </c>
       <c r="D19">
         <v>2</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="13">
         <v>10</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="14">
         <v>3.4000000000000002E-2</v>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="15">
         <f t="shared" si="0"/>
         <v>0.34</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="J19" t="s">
-        <v>115</v>
-      </c>
-      <c r="K19" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C20" t="s">
-        <v>148</v>
+        <v>107</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="D20">
         <v>2</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="12">
         <v>10</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="14">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="14">
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="J20" t="s">
-        <v>115</v>
-      </c>
-      <c r="K20" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F21" t="s">
-        <v>169</v>
-      </c>
-      <c r="G21" s="18">
+        <v>151</v>
+      </c>
+      <c r="G21" s="14">
         <f>SUM(G2:G20)</f>
         <v>130.7731</v>
       </c>
-      <c r="K21" s="20" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="K22" s="20" t="s">
-        <v>115</v>
+      <c r="K21" s="16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K22" s="16" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -3960,6 +3875,7 @@
     <hyperlink ref="L5" r:id="rId21" xr:uid="{10AA818C-D46B-2E4F-9DF0-1368C0673C54}"/>
     <hyperlink ref="J11" r:id="rId22" xr:uid="{A2FE312B-B17E-6E40-B50F-03184E20CC67}"/>
     <hyperlink ref="I12" r:id="rId23" xr:uid="{E869A8A3-1E39-324F-B9EB-AEB400CA1C48}"/>
+    <hyperlink ref="I7" r:id="rId24" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/S2B-PH-K-S/926626?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlg8DtxjqiUDwety2k6cAQ0XJ&amp;gclid=Cj0KCQjwlLDQBhDjARIsAPlIefHomTfTUoZ7D0P94S5mAVF3io454K95fTm66EAoDjt__qy-ohuCJpkaAg9wEALw_wcB" xr:uid="{58E6B9D1-8FD5-4BD0-9D16-E895003F13EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3968,891 +3884,335 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{647D274E-51ED-9340-8C08-59AC0A5619B3}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>59</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="21" t="b">
+      <c r="B2" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="18">
         <v>46160</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="21" t="b">
+      <c r="D2" s="18"/>
+      <c r="E2" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="14">
         <v>4.16</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="21" t="b">
+      <c r="B3" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="21" t="b">
+      <c r="E3" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="15">
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="21" t="b">
+      <c r="B4" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="21" t="b">
+      <c r="E4" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F4" s="18">
+      <c r="F4" s="14">
         <v>7.01</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="21" t="b">
+      <c r="B5" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="21" t="b">
+      <c r="E5" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="15">
         <v>0.75770000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="21" t="b">
+      <c r="B6" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="18">
         <v>46160</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="21" t="b">
+      <c r="D6" s="18"/>
+      <c r="E6" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="15">
         <v>1.28</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="B7" s="21" t="b">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="21" t="b">
+      <c r="E7" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="14">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="B8" s="21" t="b">
+        <v>128</v>
+      </c>
+      <c r="B8" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="21" t="b">
+      <c r="E8" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="14">
         <v>1.06</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="21" t="b">
+      <c r="B9" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="18">
         <v>46160</v>
       </c>
-      <c r="D9" s="22"/>
-      <c r="E9" s="21" t="b">
+      <c r="D9" s="18"/>
+      <c r="E9" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="14">
         <v>0.4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="21" t="b">
+      <c r="B10" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="21" t="b">
+      <c r="E10" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="14">
         <v>31.88</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="21" t="b">
+      <c r="B11" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="21" t="b">
+      <c r="E11" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="14">
         <v>1.95</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="21" t="b">
+      <c r="B12" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="21" t="b">
+      <c r="E12" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="14">
         <v>0.75</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="21" t="b">
+      <c r="B13" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="21" t="b">
+      <c r="E13" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="14">
         <v>0.92</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B14" s="21" t="b">
+        <v>125</v>
+      </c>
+      <c r="B14" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="18">
         <v>46160</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="21" t="b">
+      <c r="D14" s="18"/>
+      <c r="E14" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="14">
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="21" t="b">
+      <c r="B15" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="18">
         <v>46160</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="21" t="b">
+      <c r="D15" s="18"/>
+      <c r="E15" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="14">
         <v>0.03</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="21" t="b">
+      <c r="B16" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="18">
         <v>46160</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="21" t="b">
+      <c r="D16" s="18"/>
+      <c r="E16" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F16" s="18">
+      <c r="F16" s="14">
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="21" t="b">
+      <c r="B17" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="18">
         <v>46160</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="21" t="b">
+      <c r="D17" s="18"/>
+      <c r="E17" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F17" s="18">
+      <c r="F17" s="14">
         <v>7.1999999999999995E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B18" s="21" t="b">
+      <c r="B18" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="18">
         <v>46160</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="21" t="b">
+      <c r="D18" s="18"/>
+      <c r="E18" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="14">
         <v>0.28499999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B19" s="21" t="b">
+        <v>101</v>
+      </c>
+      <c r="B19" s="17" t="b">
         <v>1</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="18">
         <v>46160</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="21" t="b">
+      <c r="D19" s="18"/>
+      <c r="E19" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="14">
         <v>3.4000000000000002E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B20" s="21" t="b">
+        <v>107</v>
+      </c>
+      <c r="B20" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="21" t="b">
+      <c r="E20" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="14">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D2AD354-F000-43EA-9051-5CE410C07359}">
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.1640625" customWidth="1"/>
-    <col min="4" max="4" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.1640625" customWidth="1"/>
-    <col min="7" max="7" width="26.33203125" customWidth="1"/>
-    <col min="8" max="8" width="21.1640625" customWidth="1"/>
-    <col min="9" max="9" width="25.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="3"/>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="16">
-        <v>3</v>
-      </c>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="16">
-        <v>3</v>
-      </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="D4" s="16">
-        <v>3</v>
-      </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="D5" s="16">
-        <v>3</v>
-      </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D6" s="16">
-        <v>3</v>
-      </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D7" s="16">
-        <v>5</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H8" s="3"/>
-      <c r="I8" s="9" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="D9" s="16">
-        <v>3</v>
-      </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="3">
-        <v>3000</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="16">
-        <v>2</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="D11" s="16">
-        <v>3</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H11" s="3">
-        <v>1660</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="16">
-        <v>0</v>
-      </c>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="3">
-        <v>3814</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D13" s="16">
-        <v>3</v>
-      </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H13" s="3">
-        <v>1050170001</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="16">
-        <v>10</v>
-      </c>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" s="16">
-        <v>10</v>
-      </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="16">
-        <v>10</v>
-      </c>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D17" s="16">
-        <v>10</v>
-      </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D18" s="16">
-        <v>10</v>
-      </c>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D19" s="16">
-        <v>10</v>
-      </c>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="D20" s="14">
-        <v>10</v>
-      </c>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="I3" r:id="rId1" xr:uid="{31FC6B69-5789-4827-9AE6-1FDFEC130E57}"/>
-    <hyperlink ref="I4" r:id="rId2" xr:uid="{E0FF750D-FB57-494B-943F-1A5E4A5542D7}"/>
-    <hyperlink ref="I5" r:id="rId3" xr:uid="{021F043F-7EF2-496D-83EB-B16BE8D4F9BA}"/>
-    <hyperlink ref="I6" r:id="rId4" xr:uid="{D10AA4C6-E88F-4764-95EE-C25ABD0479B7}"/>
-    <hyperlink ref="I10" r:id="rId5" xr:uid="{5D0C70D4-5498-499B-865E-C60ACE6BBF8F}"/>
-    <hyperlink ref="I2" r:id="rId6" xr:uid="{8A7C3480-A083-459F-8F31-B8647CE4C022}"/>
-    <hyperlink ref="I11" r:id="rId7" xr:uid="{9A94D641-5AFC-49EC-9BF9-104905A660AB}"/>
-    <hyperlink ref="I7" r:id="rId8" xr:uid="{43CCF304-4094-5842-9C38-8C3EAA24A372}"/>
-    <hyperlink ref="C2" r:id="rId9" xr:uid="{4A284219-9C9C-8C4F-9C77-2B23FE253EF7}"/>
-    <hyperlink ref="C17" r:id="rId10" xr:uid="{BBE32052-F3D2-CA4C-A6FC-CAC6CC4119AD}"/>
-    <hyperlink ref="C12" r:id="rId11" xr:uid="{2F090D7A-C40F-A245-9BA3-E8029F119E8E}"/>
-    <hyperlink ref="C4" r:id="rId12" xr:uid="{DFC0997F-50D3-A94A-A5D1-B4F058B1C292}"/>
-    <hyperlink ref="C15" r:id="rId13" xr:uid="{1D3B6864-CCB3-034B-B689-A2E42A021B32}"/>
-    <hyperlink ref="C14" r:id="rId14" xr:uid="{74EFB29F-7F3B-1541-B20E-BB8EB894C5D4}"/>
-    <hyperlink ref="C10" r:id="rId15" display="https://www.digikey.com/en/products/detail/sparkfun-electronics/SEN-11574/5762397?utm_adgroup=Gadgets%2C%20Gizmos&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_campaign=Shopping_Product_Maker%2FDIY%2C%20Educational_NEW&amp;utm_term=&amp;utm_content=Gadgets%2C%20Gizmos&amp;gclid=CjwKCAjw9pGjBhB-EiwAa5jl3J_1Q2A72ybnR56Rk9sAeqpF2Q-o0ZcV8a4OguEqfE4Nv3m8NDQ9yxoCtdIQAvD_BwE" xr:uid="{2C80E3DB-BC28-9845-9865-6FA905F21E1F}"/>
-    <hyperlink ref="C3" r:id="rId16" xr:uid="{5F04213E-9778-DC4D-BFF7-C85811648BE8}"/>
-    <hyperlink ref="C16" r:id="rId17" xr:uid="{B448CE1F-BFFC-1D48-A067-54C36FA9D5B2}"/>
-    <hyperlink ref="C19" r:id="rId18" xr:uid="{98CD5408-3EAF-8B46-9E9E-856A3242E323}"/>
-    <hyperlink ref="C18" r:id="rId19" xr:uid="{32F13DC6-1567-A54C-8B46-F9AFE6ECD12C}"/>
-    <hyperlink ref="C20" r:id="rId20" xr:uid="{EEC7EDF7-A580-E94F-A413-D9D3C1B9B083}"/>
-    <hyperlink ref="C8" r:id="rId21" xr:uid="{E3F21928-8DA8-3841-8335-32FEA84720BE}"/>
-    <hyperlink ref="E7" r:id="rId22" xr:uid="{CE7992D0-B119-6B4C-B345-9C25EF9FE2C3}"/>
-    <hyperlink ref="E11" r:id="rId23" xr:uid="{B5C99938-5A12-5C43-B38A-88FEEC725884}"/>
-    <hyperlink ref="C13" r:id="rId24" xr:uid="{0F3CB72E-BCDA-134F-BD19-312DB2E785FD}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Added Sheet - HDK Kit
</commit_message>
<xml_diff>
--- a/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
+++ b/hardware/v0.1.1/Bill_of_materials_v0.1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidstjohn/Desktop/Edge-Computing-Power-Management-Development-Kit/hardware/v0.1.1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9DE2E0-A565-7245-A971-421DA47454FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C523EE78-AAE1-1046-974C-C76389470357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PATCH 6.0" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="PATCH 8.0A" sheetId="5" r:id="rId5"/>
     <sheet name="PATCH 8.0D" sheetId="6" r:id="rId6"/>
     <sheet name="BOM" sheetId="8" r:id="rId7"/>
-    <sheet name="Orders" sheetId="9" r:id="rId8"/>
+    <sheet name="HDK Spares Kit" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="167">
   <si>
     <t xml:space="preserve">Part </t>
   </si>
@@ -504,18 +504,6 @@
     <t>Vendo 1</t>
   </si>
   <si>
-    <t>Order Date</t>
-  </si>
-  <si>
-    <t>Arrived</t>
-  </si>
-  <si>
-    <t>Unit Price</t>
-  </si>
-  <si>
-    <t>Quantity Ordered</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.mouser.com/ProductDetail/Adafruit/1660?qs=GURawfaeGuCXDyGMVdt6Kw%3D%3D </t>
   </si>
   <si>
@@ -534,16 +522,28 @@
     <t>Vendor 4</t>
   </si>
   <si>
-    <t>No Longer Manufactured</t>
-  </si>
-  <si>
-    <t>Use Asif's</t>
-  </si>
-  <si>
-    <t>See if you can find a similar one</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.mouser.com/ProductDetail/Analog-Devices/ADXL326BCPZ-RL7?qs=WIvQP4zGanhGLfyCrKqf%252Bw%3D%3D </t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Vendor 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/en/products/detail/nxp-usa-inc/PCF8523T-1-118/2530422?s=N4IgTCBcDaIAoGEBiAOArGAzAFQPQEYAaffFEAXQF8g </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/en/products/detail/abracon-llc/ABS05-32-768KHZ-6-T/15621978?s=N4IgTCBcDaIIICEDKAGArAWgMxgHQHYA2ADgGsAJALw0IwBUQBdAXyA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.adafruit.com/product/1660?srsltid=AfmBOorrT80rcMpqkBpUUoU3cXXT8WnDFTf0aV5b-lrQjgjUIcOMFST0 </t>
+  </si>
+  <si>
+    <t>Out of stock at Mouser, but it looks like it will arrive in around a month, which shouldn't be a problem. Shipping through Adafruit would be $10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/en/products/detail/molex/1050170001/2350832?s=N4IgTCBcDaIIwAYCsC4HYC0DtxAXQF8g </t>
   </si>
 </sst>
 </file>
@@ -635,7 +635,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -671,14 +671,6 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -698,23 +690,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <bag type="Checkbox"/>
-  <bag type="XFControls">
-    <bagId k="CellControl">0</bagId>
-  </bag>
-  <bag type="XFComplement">
-    <bagId k="XFControls">1</bagId>
-  </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
-</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3215,7 +3190,7 @@
         <v>149</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
@@ -3225,7 +3200,7 @@
       <c r="B2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="17" t="s">
         <v>65</v>
       </c>
       <c r="D2">
@@ -3311,13 +3286,13 @@
         <v>91</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="K4" s="8" t="s">
         <v>148</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="M4" s="8" t="s">
         <v>106</v>
@@ -3347,7 +3322,7 @@
         <v>2.2731000000000003</v>
       </c>
       <c r="H5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>111</v>
@@ -3359,7 +3334,7 @@
         <v>150</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="M5" t="s">
         <v>106</v>
@@ -3415,14 +3390,14 @@
         <v>5</v>
       </c>
       <c r="F7" s="14">
-        <v>1.1000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="G7" s="15">
         <f t="shared" si="0"/>
-        <v>5.5</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>106</v>
@@ -3557,7 +3532,7 @@
         <v>114</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>106</v>
@@ -3866,7 +3841,7 @@
       </c>
       <c r="G21" s="14">
         <f>SUM(G2:G20)</f>
-        <v>130.7731</v>
+        <v>125.8231</v>
       </c>
       <c r="K21" s="16" t="s">
         <v>106</v>
@@ -3912,380 +3887,219 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{647D274E-51ED-9340-8C08-59AC0A5619B3}">
-  <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15166C97-981B-954B-AAC2-0255786EEB41}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>153</v>
+        <v>122</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>154</v>
+        <v>120</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>155</v>
+        <v>161</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="17" t="b">
+      <c r="C2" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2" s="14">
+        <v>4.16</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="G2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="C2" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" s="14">
-        <v>4.16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" s="18">
-        <v>46167</v>
-      </c>
-      <c r="E3" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" s="15">
-        <v>0.57999999999999996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="18">
-        <v>46167</v>
-      </c>
-      <c r="E4" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>165</v>
+      <c r="E4" s="14">
+        <v>1.35</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="G4" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" s="18">
-        <v>46166</v>
-      </c>
-      <c r="E5" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="15">
-        <v>0.75770000000000004</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" s="14">
+        <v>1.28</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>163</v>
       </c>
+      <c r="G5" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="18">
-        <v>46160</v>
+      <c r="A6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="3">
+        <v>9749</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
-      <c r="E6" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" s="15">
-        <v>1.28</v>
+      <c r="E6" s="14">
+        <v>0.11</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="G6" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="B7" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="18">
-        <v>46166</v>
-      </c>
-      <c r="E7" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14">
-        <v>1.1000000000000001</v>
+      <c r="A7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1660</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1.95</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H7" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B8" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="18">
-        <v>46166</v>
-      </c>
-      <c r="E8" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14">
-        <v>1.06</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" s="14">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F10" s="14">
-        <v>31.88</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C11" s="18">
-        <v>46166</v>
-      </c>
-      <c r="E11" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" s="14">
-        <v>1.95</v>
-      </c>
-      <c r="H11" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" s="18">
-        <v>46167</v>
-      </c>
-      <c r="E12" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" s="14">
+      <c r="C8" s="3">
+        <v>1050170001</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" s="14">
         <v>0.92</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B13" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D13">
-        <v>10</v>
-      </c>
-      <c r="E13" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" s="14">
-        <v>2.1000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C14" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D14">
-        <v>10</v>
-      </c>
-      <c r="E14" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" s="14">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D15">
-        <v>10</v>
-      </c>
-      <c r="E15" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F15" s="14">
-        <v>3.6999999999999998E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C16" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D16">
-        <v>10</v>
-      </c>
-      <c r="E16" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" s="14">
-        <v>7.1999999999999995E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C17" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D17">
-        <v>10</v>
-      </c>
-      <c r="E17" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" s="14">
-        <v>0.28499999999999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B18" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C18" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D18">
-        <v>10</v>
-      </c>
-      <c r="E18" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" s="14">
-        <v>3.4000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B19" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19" s="18">
-        <v>46160</v>
-      </c>
-      <c r="D19">
-        <v>10</v>
-      </c>
-      <c r="E19" s="17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" s="14">
-        <v>2.5000000000000001E-2</v>
+      <c r="F8" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="G8" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{8848112D-74EB-AD46-9468-10EF10A47D55}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{6911CFEE-0308-1948-83C3-DF19A8B4E8BF}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{CEBA6C16-0C1F-C344-A732-C45D5C9FC6FC}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{94889B94-DDBF-3F49-BA60-587DAABBB279}"/>
+    <hyperlink ref="F6" r:id="rId5" display="https://www.digikey.com/en/products/detail/jst-sales-america-inc/S2B-PH-K-S/926626?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20470400566&amp;gbraid=0AAAAADrbLlg8DtxjqiUDwety2k6cAQ0XJ&amp;gclid=Cj0KCQjwlLDQBhDjARIsAPlIefHomTfTUoZ7D0P94S5mAVF3io454K95fTm66EAoDjt__qy-ohuCJpkaAg9wEALw_wcB" xr:uid="{53BFEA82-54D5-974F-9085-E4AA3562A5FC}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{D47423DA-5F73-8D42-AF7E-9C5B70B654FD}"/>
+    <hyperlink ref="F7" r:id="rId7" xr:uid="{17098019-0BD5-6C4F-9DC4-DEA8DBA7D649}"/>
+    <hyperlink ref="F8" r:id="rId8" xr:uid="{93CFCB2E-079C-FD45-B36B-E6607FB5CC3F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>